<commit_message>
E4: datos de ejemplo, archivos ficticios de v3, pruebas con un comando y acción de pruebas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USu2EeotXdexQTeeRTuiif
</commit_message>
<xml_diff>
--- a/datos-demo/v3-prueba.xlsx
+++ b/datos-demo/v3-prueba.xlsx
@@ -704,6 +704,15 @@
       <c r="AC3" t="n">
         <v>50000</v>
       </c>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>200</v>
+      </c>
       <c r="AP3" t="inlineStr">
         <is>
           <t>💰 Ingreso</t>
@@ -737,6 +746,15 @@
       <c r="AC4" t="n">
         <v>150000</v>
       </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>200</v>
+      </c>
       <c r="AP4" t="inlineStr">
         <is>
           <t>💰 Ingreso</t>
@@ -770,6 +788,15 @@
       <c r="AC5" t="n">
         <v>120000</v>
       </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>200</v>
+      </c>
       <c r="AP5" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -806,6 +833,15 @@
       <c r="AC6" t="n">
         <v>120000</v>
       </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>200</v>
+      </c>
       <c r="AP6" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -839,6 +875,15 @@
       <c r="AC7" t="n">
         <v>120000</v>
       </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>200</v>
+      </c>
       <c r="AP7" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -872,6 +917,15 @@
       <c r="AC8" t="n">
         <v>120000</v>
       </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>200</v>
+      </c>
       <c r="AP8" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -905,6 +959,15 @@
       <c r="AC9" t="n">
         <v>120000</v>
       </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>200</v>
+      </c>
       <c r="AP9" t="inlineStr">
         <is>
           <t>🔄 Transacción entre las billeteras</t>
@@ -935,8 +998,17 @@
       <c r="AC10" t="n">
         <v>120000</v>
       </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
       <c r="AL10" t="n">
         <v>100</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>300</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
@@ -968,8 +1040,17 @@
       <c r="AC11" t="n">
         <v>120000</v>
       </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
       <c r="AM11" t="n">
         <v>50</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>250</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
@@ -1012,6 +1093,15 @@
       <c r="AE12" t="n">
         <v>15000</v>
       </c>
+      <c r="AG12" t="n">
+        <v>15000</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>250</v>
+      </c>
       <c r="AP12" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -1053,6 +1143,15 @@
       <c r="AF13" t="n">
         <v>15000</v>
       </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>250</v>
+      </c>
       <c r="AP13" t="inlineStr">
         <is>
           <t>💰 Ingreso</t>
@@ -1086,6 +1185,9 @@
       <c r="AC14" t="n">
         <v>128000</v>
       </c>
+      <c r="AG14" t="n">
+        <v>0</v>
+      </c>
       <c r="AH14" t="inlineStr">
         <is>
           <t>Persona B</t>
@@ -1093,6 +1195,12 @@
       </c>
       <c r="AJ14" t="n">
         <v>8000</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>250</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
@@ -1127,6 +1235,9 @@
       <c r="AC15" t="n">
         <v>120000</v>
       </c>
+      <c r="AG15" t="n">
+        <v>0</v>
+      </c>
       <c r="AH15" t="inlineStr">
         <is>
           <t>Persona B</t>
@@ -1134,6 +1245,12 @@
       </c>
       <c r="AI15" t="n">
         <v>8000</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>250</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
@@ -1168,6 +1285,15 @@
       <c r="AC16" t="n">
         <v>120000</v>
       </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>250</v>
+      </c>
       <c r="AP16" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -1201,6 +1327,15 @@
       <c r="AC17" t="n">
         <v>120000</v>
       </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>250</v>
+      </c>
       <c r="AP17" t="inlineStr">
         <is>
           <t>💰 Ingreso</t>
@@ -1234,6 +1369,15 @@
       <c r="AC18" t="n">
         <v>121200</v>
       </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>250</v>
+      </c>
       <c r="AP18" t="inlineStr">
         <is>
           <t>💰 Ingreso</t>
@@ -1267,6 +1411,15 @@
       <c r="AC19" t="n">
         <v>109200</v>
       </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1292,6 +1445,15 @@
       <c r="AC20" t="n">
         <v>109200</v>
       </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>250</v>
+      </c>
       <c r="AP20" t="inlineStr">
         <is>
           <t>💸 Egreso</t>
@@ -1317,6 +1479,15 @@
       <c r="AC21" t="n">
         <v>109200</v>
       </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1345,6 +1516,15 @@
       <c r="AC22" t="n">
         <v>109200</v>
       </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>250</v>
+      </c>
       <c r="AP22" t="inlineStr">
         <is>
           <t>💰 Ingreso</t>
@@ -1377,6 +1557,15 @@
       </c>
       <c r="AC23" t="n">
         <v>109200</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>250</v>
       </c>
       <c r="AP23" t="inlineStr">
         <is>

</xml_diff>